<commit_message>
Fixed big and models
</commit_message>
<xml_diff>
--- a/val_predictions.xlsx
+++ b/val_predictions.xlsx
@@ -467,16 +467,16 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>1.63</v>
+        <v>1.590000033378601</v>
       </c>
       <c r="C2" t="n">
-        <v>1.5</v>
+        <v>2.200000047683716</v>
       </c>
       <c r="D2" t="n">
-        <v>1.54</v>
+        <v>1.649999976158142</v>
       </c>
       <c r="E2" t="n">
-        <v>4.67</v>
+        <v>5.440000057220459</v>
       </c>
       <c r="F2" t="n">
         <v>0</v>
@@ -489,16 +489,16 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>1.46</v>
+        <v>1.570000052452087</v>
       </c>
       <c r="C3" t="n">
-        <v>0.71</v>
+        <v>1.370000004768372</v>
       </c>
       <c r="D3" t="n">
-        <v>2.03</v>
+        <v>2.210000038146973</v>
       </c>
       <c r="E3" t="n">
-        <v>4.2</v>
+        <v>5.150000095367432</v>
       </c>
       <c r="F3" t="n">
         <v>0</v>
@@ -511,19 +511,19 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>1.59</v>
+        <v>1.539999961853027</v>
       </c>
       <c r="C4" t="n">
-        <v>2.14</v>
+        <v>2.140000104904175</v>
       </c>
       <c r="D4" t="n">
-        <v>2.44</v>
+        <v>2.109999895095825</v>
       </c>
       <c r="E4" t="n">
-        <v>6.17</v>
+        <v>5.789999961853027</v>
       </c>
       <c r="F4" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="5">
@@ -533,16 +533,16 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>1.87</v>
+        <v>1.480000019073486</v>
       </c>
       <c r="C5" t="n">
-        <v>1.9</v>
+        <v>1.850000023841858</v>
       </c>
       <c r="D5" t="n">
-        <v>1.91</v>
+        <v>1.879999995231628</v>
       </c>
       <c r="E5" t="n">
-        <v>5.68</v>
+        <v>5.210000038146973</v>
       </c>
       <c r="F5" t="n">
         <v>0</v>
@@ -555,19 +555,19 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>1.88</v>
+        <v>1.309999942779541</v>
       </c>
       <c r="C6" t="n">
-        <v>2.18</v>
+        <v>1.830000042915344</v>
       </c>
       <c r="D6" t="n">
-        <v>2.72</v>
+        <v>2.200000047683716</v>
       </c>
       <c r="E6" t="n">
-        <v>6.78</v>
+        <v>5.340000152587891</v>
       </c>
       <c r="F6" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="7">
@@ -577,16 +577,16 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>0.78</v>
+        <v>0.75</v>
       </c>
       <c r="C7" t="n">
-        <v>2.36</v>
+        <v>1.590000033378601</v>
       </c>
       <c r="D7" t="n">
-        <v>2.22</v>
+        <v>2.25</v>
       </c>
       <c r="E7" t="n">
-        <v>5.36</v>
+        <v>4.590000152587891</v>
       </c>
       <c r="F7" t="n">
         <v>0</v>
@@ -599,16 +599,16 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>1.99</v>
+        <v>2.069999933242798</v>
       </c>
       <c r="C8" t="n">
-        <v>2.33</v>
+        <v>2.759999990463257</v>
       </c>
       <c r="D8" t="n">
-        <v>2.13</v>
+        <v>2.529999971389771</v>
       </c>
       <c r="E8" t="n">
-        <v>6.45</v>
+        <v>7.360000133514404</v>
       </c>
       <c r="F8" t="n">
         <v>1</v>
@@ -621,19 +621,19 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>2.66</v>
+        <v>1.559999942779541</v>
       </c>
       <c r="C9" t="n">
-        <v>2.35</v>
+        <v>2.140000104904175</v>
       </c>
       <c r="D9" t="n">
-        <v>2.22</v>
+        <v>2.259999990463257</v>
       </c>
       <c r="E9" t="n">
-        <v>7.23</v>
+        <v>5.960000038146973</v>
       </c>
       <c r="F9" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="10">
@@ -643,16 +643,16 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>2.02</v>
+        <v>2.299999952316284</v>
       </c>
       <c r="C10" t="n">
-        <v>2.69</v>
+        <v>3</v>
       </c>
       <c r="D10" t="n">
-        <v>2.52</v>
+        <v>2.440000057220459</v>
       </c>
       <c r="E10" t="n">
-        <v>7.23</v>
+        <v>7.739999771118164</v>
       </c>
       <c r="F10" t="n">
         <v>1</v>
@@ -665,16 +665,16 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>0.91</v>
+        <v>0.4900000095367432</v>
       </c>
       <c r="C11" t="n">
-        <v>0.87</v>
+        <v>0.9300000071525574</v>
       </c>
       <c r="D11" t="n">
-        <v>2.18</v>
+        <v>2.079999923706055</v>
       </c>
       <c r="E11" t="n">
-        <v>3.96</v>
+        <v>3.5</v>
       </c>
       <c r="F11" t="n">
         <v>0</v>
@@ -687,16 +687,16 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>1.42</v>
+        <v>1</v>
       </c>
       <c r="C12" t="n">
-        <v>1.25</v>
+        <v>1.850000023841858</v>
       </c>
       <c r="D12" t="n">
-        <v>0.84</v>
+        <v>0.2199999988079071</v>
       </c>
       <c r="E12" t="n">
-        <v>3.51</v>
+        <v>3.069999933242798</v>
       </c>
       <c r="F12" t="n">
         <v>0</v>
@@ -709,16 +709,16 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>1.05</v>
+        <v>1.269999980926514</v>
       </c>
       <c r="C13" t="n">
-        <v>0.96</v>
+        <v>1.570000052452087</v>
       </c>
       <c r="D13" t="n">
-        <v>1.63</v>
+        <v>1.230000019073486</v>
       </c>
       <c r="E13" t="n">
-        <v>3.64</v>
+        <v>4.070000171661377</v>
       </c>
       <c r="F13" t="n">
         <v>0</v>
@@ -731,16 +731,16 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>0.78</v>
+        <v>0.3400000035762787</v>
       </c>
       <c r="C14" t="n">
-        <v>0.95</v>
+        <v>0.8399999737739563</v>
       </c>
       <c r="D14" t="n">
-        <v>1.11</v>
+        <v>0.8999999761581421</v>
       </c>
       <c r="E14" t="n">
-        <v>2.84</v>
+        <v>2.079999923706055</v>
       </c>
       <c r="F14" t="n">
         <v>0</v>
@@ -753,16 +753,16 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>0.99</v>
+        <v>1.110000014305115</v>
       </c>
       <c r="C15" t="n">
-        <v>1.44</v>
+        <v>1.720000028610229</v>
       </c>
       <c r="D15" t="n">
-        <v>1.97</v>
+        <v>2.329999923706055</v>
       </c>
       <c r="E15" t="n">
-        <v>4.4</v>
+        <v>5.159999847412109</v>
       </c>
       <c r="F15" t="n">
         <v>0</v>
@@ -775,19 +775,19 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>1.72</v>
+        <v>1.389999985694885</v>
       </c>
       <c r="C16" t="n">
-        <v>2.23</v>
+        <v>2.460000038146973</v>
       </c>
       <c r="D16" t="n">
-        <v>2.4</v>
+        <v>2.099999904632568</v>
       </c>
       <c r="E16" t="n">
-        <v>6.35</v>
+        <v>5.949999809265137</v>
       </c>
       <c r="F16" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="17">
@@ -797,16 +797,16 @@
         </is>
       </c>
       <c r="B17" t="n">
-        <v>0.34</v>
+        <v>0.03999999910593033</v>
       </c>
       <c r="C17" t="n">
-        <v>0.95</v>
+        <v>0.7099999785423279</v>
       </c>
       <c r="D17" t="n">
-        <v>1.59</v>
+        <v>1.659999966621399</v>
       </c>
       <c r="E17" t="n">
-        <v>2.88</v>
+        <v>2.410000085830688</v>
       </c>
       <c r="F17" t="n">
         <v>0</v>
@@ -819,16 +819,16 @@
         </is>
       </c>
       <c r="B18" t="n">
-        <v>1.2</v>
+        <v>0.8999999761581421</v>
       </c>
       <c r="C18" t="n">
-        <v>1.77</v>
+        <v>2</v>
       </c>
       <c r="D18" t="n">
-        <v>0.57</v>
+        <v>0.949999988079071</v>
       </c>
       <c r="E18" t="n">
-        <v>3.54</v>
+        <v>3.849999904632568</v>
       </c>
       <c r="F18" t="n">
         <v>0</v>
@@ -841,16 +841,16 @@
         </is>
       </c>
       <c r="B19" t="n">
-        <v>2.17</v>
+        <v>2.450000047683716</v>
       </c>
       <c r="C19" t="n">
-        <v>2.36</v>
+        <v>2.710000038146973</v>
       </c>
       <c r="D19" t="n">
-        <v>2.92</v>
+        <v>2.569999933242798</v>
       </c>
       <c r="E19" t="n">
-        <v>7.45</v>
+        <v>7.730000019073486</v>
       </c>
       <c r="F19" t="n">
         <v>1</v>
@@ -863,16 +863,16 @@
         </is>
       </c>
       <c r="B20" t="n">
-        <v>1.14</v>
+        <v>1.730000019073486</v>
       </c>
       <c r="C20" t="n">
-        <v>2.2</v>
+        <v>2.440000057220459</v>
       </c>
       <c r="D20" t="n">
-        <v>1.66</v>
+        <v>1.379999995231628</v>
       </c>
       <c r="E20" t="n">
-        <v>5</v>
+        <v>5.550000190734863</v>
       </c>
       <c r="F20" t="n">
         <v>0</v>
@@ -885,16 +885,16 @@
         </is>
       </c>
       <c r="B21" t="n">
-        <v>1.61</v>
+        <v>1.919999957084656</v>
       </c>
       <c r="C21" t="n">
-        <v>1.96</v>
+        <v>1.990000009536743</v>
       </c>
       <c r="D21" t="n">
-        <v>2.62</v>
+        <v>2.660000085830688</v>
       </c>
       <c r="E21" t="n">
-        <v>6.19</v>
+        <v>6.570000171661377</v>
       </c>
       <c r="F21" t="n">
         <v>1</v>
@@ -907,16 +907,16 @@
         </is>
       </c>
       <c r="B22" t="n">
-        <v>0.44</v>
+        <v>0.6800000071525574</v>
       </c>
       <c r="C22" t="n">
-        <v>1.67</v>
+        <v>1.429999947547913</v>
       </c>
       <c r="D22" t="n">
-        <v>1.5</v>
+        <v>1.299999952316284</v>
       </c>
       <c r="E22" t="n">
-        <v>3.61</v>
+        <v>3.410000085830688</v>
       </c>
       <c r="F22" t="n">
         <v>0</v>
@@ -929,16 +929,16 @@
         </is>
       </c>
       <c r="B23" t="n">
-        <v>1.2</v>
+        <v>1.179999947547913</v>
       </c>
       <c r="C23" t="n">
-        <v>2.09</v>
+        <v>2.130000114440918</v>
       </c>
       <c r="D23" t="n">
-        <v>1.98</v>
+        <v>2.609999895095825</v>
       </c>
       <c r="E23" t="n">
-        <v>5.27</v>
+        <v>5.920000076293945</v>
       </c>
       <c r="F23" t="n">
         <v>0</v>
@@ -951,16 +951,16 @@
         </is>
       </c>
       <c r="B24" t="n">
-        <v>1.74</v>
+        <v>1.980000019073486</v>
       </c>
       <c r="C24" t="n">
-        <v>2.11</v>
+        <v>2.130000114440918</v>
       </c>
       <c r="D24" t="n">
-        <v>2.35</v>
+        <v>2.369999885559082</v>
       </c>
       <c r="E24" t="n">
-        <v>6.2</v>
+        <v>6.480000019073486</v>
       </c>
       <c r="F24" t="n">
         <v>1</v>
@@ -973,16 +973,16 @@
         </is>
       </c>
       <c r="B25" t="n">
-        <v>1.53</v>
+        <v>1.529999971389771</v>
       </c>
       <c r="C25" t="n">
-        <v>1.72</v>
+        <v>1.529999971389771</v>
       </c>
       <c r="D25" t="n">
-        <v>2.07</v>
+        <v>1.850000023841858</v>
       </c>
       <c r="E25" t="n">
-        <v>5.32</v>
+        <v>4.909999847412109</v>
       </c>
       <c r="F25" t="n">
         <v>0</v>
@@ -995,16 +995,16 @@
         </is>
       </c>
       <c r="B26" t="n">
-        <v>2.33</v>
+        <v>2.109999895095825</v>
       </c>
       <c r="C26" t="n">
-        <v>2.76</v>
+        <v>1.970000028610229</v>
       </c>
       <c r="D26" t="n">
-        <v>2.54</v>
+        <v>2.210000038146973</v>
       </c>
       <c r="E26" t="n">
-        <v>7.63</v>
+        <v>6.289999961853027</v>
       </c>
       <c r="F26" t="n">
         <v>1</v>
@@ -1017,16 +1017,16 @@
         </is>
       </c>
       <c r="B27" t="n">
-        <v>0.91</v>
+        <v>1.039999961853027</v>
       </c>
       <c r="C27" t="n">
-        <v>1.23</v>
+        <v>1.129999995231628</v>
       </c>
       <c r="D27" t="n">
-        <v>2.02</v>
+        <v>2.210000038146973</v>
       </c>
       <c r="E27" t="n">
-        <v>4.16</v>
+        <v>4.380000114440918</v>
       </c>
       <c r="F27" t="n">
         <v>0</v>
@@ -1039,16 +1039,16 @@
         </is>
       </c>
       <c r="B28" t="n">
-        <v>1.29</v>
+        <v>1.019999980926514</v>
       </c>
       <c r="C28" t="n">
-        <v>1.66</v>
+        <v>1.889999985694885</v>
       </c>
       <c r="D28" t="n">
-        <v>2</v>
+        <v>1.620000004768372</v>
       </c>
       <c r="E28" t="n">
-        <v>4.95</v>
+        <v>4.53000020980835</v>
       </c>
       <c r="F28" t="n">
         <v>0</v>
@@ -1061,16 +1061,16 @@
         </is>
       </c>
       <c r="B29" t="n">
-        <v>1.17</v>
+        <v>1.240000009536743</v>
       </c>
       <c r="C29" t="n">
-        <v>1.45</v>
+        <v>1.970000028610229</v>
       </c>
       <c r="D29" t="n">
-        <v>1.2</v>
+        <v>0.9200000166893005</v>
       </c>
       <c r="E29" t="n">
-        <v>3.82</v>
+        <v>4.130000114440918</v>
       </c>
       <c r="F29" t="n">
         <v>0</v>
@@ -1083,19 +1083,19 @@
         </is>
       </c>
       <c r="B30" t="n">
-        <v>1.4</v>
+        <v>1.399999976158142</v>
       </c>
       <c r="C30" t="n">
-        <v>2.22</v>
+        <v>1.970000028610229</v>
       </c>
       <c r="D30" t="n">
-        <v>2.74</v>
+        <v>2.440000057220459</v>
       </c>
       <c r="E30" t="n">
-        <v>6.36</v>
+        <v>5.809999942779541</v>
       </c>
       <c r="F30" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="31">
@@ -1105,16 +1105,16 @@
         </is>
       </c>
       <c r="B31" t="n">
-        <v>1.94</v>
+        <v>1.590000033378601</v>
       </c>
       <c r="C31" t="n">
-        <v>1.66</v>
+        <v>1.820000052452087</v>
       </c>
       <c r="D31" t="n">
-        <v>2.11</v>
+        <v>1.759999990463257</v>
       </c>
       <c r="E31" t="n">
-        <v>5.71</v>
+        <v>5.170000076293945</v>
       </c>
       <c r="F31" t="n">
         <v>0</v>
@@ -1127,16 +1127,16 @@
         </is>
       </c>
       <c r="B32" t="n">
-        <v>1.25</v>
+        <v>1.100000023841858</v>
       </c>
       <c r="C32" t="n">
-        <v>0.98</v>
+        <v>0.05000000074505806</v>
       </c>
       <c r="D32" t="n">
-        <v>1.12</v>
+        <v>0.9200000166893005</v>
       </c>
       <c r="E32" t="n">
-        <v>3.35</v>
+        <v>2.069999933242798</v>
       </c>
       <c r="F32" t="n">
         <v>0</v>
@@ -1149,16 +1149,16 @@
         </is>
       </c>
       <c r="B33" t="n">
-        <v>0.6</v>
+        <v>0.2300000041723251</v>
       </c>
       <c r="C33" t="n">
-        <v>0.55</v>
+        <v>0.03999999910593033</v>
       </c>
       <c r="D33" t="n">
-        <v>1.21</v>
+        <v>0.6000000238418579</v>
       </c>
       <c r="E33" t="n">
-        <v>2.36</v>
+        <v>0.8700000047683716</v>
       </c>
       <c r="F33" t="n">
         <v>0</v>
@@ -1171,16 +1171,16 @@
         </is>
       </c>
       <c r="B34" t="n">
-        <v>1.27</v>
+        <v>1.519999980926514</v>
       </c>
       <c r="C34" t="n">
-        <v>1.13</v>
+        <v>1.759999990463257</v>
       </c>
       <c r="D34" t="n">
-        <v>2.34</v>
+        <v>2.359999895095825</v>
       </c>
       <c r="E34" t="n">
-        <v>4.74</v>
+        <v>5.639999866485596</v>
       </c>
       <c r="F34" t="n">
         <v>0</v>
@@ -1193,16 +1193,16 @@
         </is>
       </c>
       <c r="B35" t="n">
-        <v>2.28</v>
+        <v>2.359999895095825</v>
       </c>
       <c r="C35" t="n">
-        <v>2.04</v>
+        <v>2.269999980926514</v>
       </c>
       <c r="D35" t="n">
-        <v>1.91</v>
+        <v>1.440000057220459</v>
       </c>
       <c r="E35" t="n">
-        <v>6.23</v>
+        <v>6.070000171661377</v>
       </c>
       <c r="F35" t="n">
         <v>1</v>
@@ -1215,16 +1215,16 @@
         </is>
       </c>
       <c r="B36" t="n">
-        <v>0.97</v>
+        <v>1</v>
       </c>
       <c r="C36" t="n">
-        <v>1.54</v>
+        <v>1.600000023841858</v>
       </c>
       <c r="D36" t="n">
-        <v>2.43</v>
+        <v>1.940000057220459</v>
       </c>
       <c r="E36" t="n">
-        <v>4.94</v>
+        <v>4.539999961853027</v>
       </c>
       <c r="F36" t="n">
         <v>0</v>
@@ -1237,16 +1237,16 @@
         </is>
       </c>
       <c r="B37" t="n">
-        <v>1.27</v>
+        <v>1.379999995231628</v>
       </c>
       <c r="C37" t="n">
-        <v>1.9</v>
+        <v>1.779999971389771</v>
       </c>
       <c r="D37" t="n">
-        <v>1.9</v>
+        <v>1.879999995231628</v>
       </c>
       <c r="E37" t="n">
-        <v>5.07</v>
+        <v>5.039999961853027</v>
       </c>
       <c r="F37" t="n">
         <v>0</v>
@@ -1259,16 +1259,16 @@
         </is>
       </c>
       <c r="B38" t="n">
-        <v>2.03</v>
+        <v>1.929999947547913</v>
       </c>
       <c r="C38" t="n">
-        <v>2.04</v>
+        <v>1.860000014305115</v>
       </c>
       <c r="D38" t="n">
-        <v>2.32</v>
+        <v>2.289999961853027</v>
       </c>
       <c r="E38" t="n">
-        <v>6.39</v>
+        <v>6.079999923706055</v>
       </c>
       <c r="F38" t="n">
         <v>1</v>
@@ -1281,16 +1281,16 @@
         </is>
       </c>
       <c r="B39" t="n">
-        <v>0.79</v>
+        <v>0.9900000095367432</v>
       </c>
       <c r="C39" t="n">
-        <v>0.98</v>
+        <v>0.8600000143051147</v>
       </c>
       <c r="D39" t="n">
-        <v>1.05</v>
+        <v>1.090000033378601</v>
       </c>
       <c r="E39" t="n">
-        <v>2.82</v>
+        <v>2.940000057220459</v>
       </c>
       <c r="F39" t="n">
         <v>0</v>
@@ -1303,16 +1303,16 @@
         </is>
       </c>
       <c r="B40" t="n">
-        <v>2.83</v>
+        <v>2.75</v>
       </c>
       <c r="C40" t="n">
-        <v>2.23</v>
+        <v>2.420000076293945</v>
       </c>
       <c r="D40" t="n">
-        <v>2.18</v>
+        <v>2.319999933242798</v>
       </c>
       <c r="E40" t="n">
-        <v>7.24</v>
+        <v>7.489999771118164</v>
       </c>
       <c r="F40" t="n">
         <v>1</v>
@@ -1325,16 +1325,16 @@
         </is>
       </c>
       <c r="B41" t="n">
-        <v>1.28</v>
+        <v>1.309999942779541</v>
       </c>
       <c r="C41" t="n">
-        <v>1.83</v>
+        <v>0.8899999856948853</v>
       </c>
       <c r="D41" t="n">
-        <v>1.46</v>
+        <v>1.200000047683716</v>
       </c>
       <c r="E41" t="n">
-        <v>4.57</v>
+        <v>3.400000095367432</v>
       </c>
       <c r="F41" t="n">
         <v>0</v>
@@ -1347,16 +1347,16 @@
         </is>
       </c>
       <c r="B42" t="n">
-        <v>1.13</v>
+        <v>1.039999961853027</v>
       </c>
       <c r="C42" t="n">
-        <v>1.84</v>
+        <v>1.379999995231628</v>
       </c>
       <c r="D42" t="n">
-        <v>1.77</v>
+        <v>1.860000014305115</v>
       </c>
       <c r="E42" t="n">
-        <v>4.74</v>
+        <v>4.28000020980835</v>
       </c>
       <c r="F42" t="n">
         <v>0</v>
@@ -1369,19 +1369,19 @@
         </is>
       </c>
       <c r="B43" t="n">
-        <v>1.96</v>
+        <v>1.399999976158142</v>
       </c>
       <c r="C43" t="n">
-        <v>1.63</v>
+        <v>1.629999995231628</v>
       </c>
       <c r="D43" t="n">
-        <v>2.57</v>
+        <v>2.130000114440918</v>
       </c>
       <c r="E43" t="n">
-        <v>6.16</v>
+        <v>5.159999847412109</v>
       </c>
       <c r="F43" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="44">
@@ -1391,16 +1391,16 @@
         </is>
       </c>
       <c r="B44" t="n">
-        <v>1.53</v>
+        <v>2.150000095367432</v>
       </c>
       <c r="C44" t="n">
-        <v>2.12</v>
+        <v>2.339999914169312</v>
       </c>
       <c r="D44" t="n">
-        <v>2.44</v>
+        <v>1.940000057220459</v>
       </c>
       <c r="E44" t="n">
-        <v>6.09</v>
+        <v>6.429999828338623</v>
       </c>
       <c r="F44" t="n">
         <v>1</v>
@@ -1413,16 +1413,16 @@
         </is>
       </c>
       <c r="B45" t="n">
-        <v>3</v>
+        <v>2.319999933242798</v>
       </c>
       <c r="C45" t="n">
-        <v>2.86</v>
+        <v>2.430000066757202</v>
       </c>
       <c r="D45" t="n">
-        <v>1.3</v>
+        <v>1.600000023841858</v>
       </c>
       <c r="E45" t="n">
-        <v>7.16</v>
+        <v>6.349999904632568</v>
       </c>
       <c r="F45" t="n">
         <v>1</v>
@@ -1435,16 +1435,16 @@
         </is>
       </c>
       <c r="B46" t="n">
-        <v>0.91</v>
+        <v>1.720000028610229</v>
       </c>
       <c r="C46" t="n">
-        <v>2.03</v>
+        <v>1.620000004768372</v>
       </c>
       <c r="D46" t="n">
-        <v>1.95</v>
+        <v>1.960000038146973</v>
       </c>
       <c r="E46" t="n">
-        <v>4.89</v>
+        <v>5.300000190734863</v>
       </c>
       <c r="F46" t="n">
         <v>0</v>
@@ -1457,16 +1457,16 @@
         </is>
       </c>
       <c r="B47" t="n">
-        <v>1.12</v>
+        <v>1.230000019073486</v>
       </c>
       <c r="C47" t="n">
-        <v>1.98</v>
+        <v>1.659999966621399</v>
       </c>
       <c r="D47" t="n">
-        <v>1.69</v>
+        <v>2.150000095367432</v>
       </c>
       <c r="E47" t="n">
-        <v>4.79</v>
+        <v>5.039999961853027</v>
       </c>
       <c r="F47" t="n">
         <v>0</v>
@@ -1479,16 +1479,16 @@
         </is>
       </c>
       <c r="B48" t="n">
-        <v>0.43</v>
+        <v>0.9300000071525574</v>
       </c>
       <c r="C48" t="n">
-        <v>0.82</v>
+        <v>0.7099999785423279</v>
       </c>
       <c r="D48" t="n">
-        <v>0.86</v>
+        <v>0.5699999928474426</v>
       </c>
       <c r="E48" t="n">
-        <v>2.11</v>
+        <v>2.210000038146973</v>
       </c>
       <c r="F48" t="n">
         <v>0</v>
@@ -1501,16 +1501,16 @@
         </is>
       </c>
       <c r="B49" t="n">
-        <v>0.24</v>
+        <v>0.1500000059604645</v>
       </c>
       <c r="C49" t="n">
-        <v>1.11</v>
+        <v>0.4799999892711639</v>
       </c>
       <c r="D49" t="n">
-        <v>1.46</v>
+        <v>0.8299999833106995</v>
       </c>
       <c r="E49" t="n">
-        <v>2.81</v>
+        <v>1.460000038146973</v>
       </c>
       <c r="F49" t="n">
         <v>0</v>
@@ -1523,16 +1523,16 @@
         </is>
       </c>
       <c r="B50" t="n">
-        <v>0.76</v>
+        <v>0.2700000107288361</v>
       </c>
       <c r="C50" t="n">
-        <v>0.83</v>
+        <v>0.6299999952316284</v>
       </c>
       <c r="D50" t="n">
-        <v>0.6899999999999999</v>
+        <v>0.7900000214576721</v>
       </c>
       <c r="E50" t="n">
-        <v>2.28</v>
+        <v>1.690000057220459</v>
       </c>
       <c r="F50" t="n">
         <v>0</v>
@@ -1545,16 +1545,16 @@
         </is>
       </c>
       <c r="B51" t="n">
-        <v>0.64</v>
+        <v>0.7200000286102295</v>
       </c>
       <c r="C51" t="n">
-        <v>1.61</v>
+        <v>2.069999933242798</v>
       </c>
       <c r="D51" t="n">
-        <v>1.73</v>
+        <v>1.740000009536743</v>
       </c>
       <c r="E51" t="n">
-        <v>3.98</v>
+        <v>4.53000020980835</v>
       </c>
       <c r="F51" t="n">
         <v>0</v>
@@ -1567,16 +1567,16 @@
         </is>
       </c>
       <c r="B52" t="n">
-        <v>2.31</v>
+        <v>2.019999980926514</v>
       </c>
       <c r="C52" t="n">
-        <v>2.09</v>
+        <v>2.220000028610229</v>
       </c>
       <c r="D52" t="n">
-        <v>0.52</v>
+        <v>1.360000014305115</v>
       </c>
       <c r="E52" t="n">
-        <v>4.92</v>
+        <v>5.599999904632568</v>
       </c>
       <c r="F52" t="n">
         <v>0</v>
@@ -1589,16 +1589,16 @@
         </is>
       </c>
       <c r="B53" t="n">
-        <v>1.73</v>
+        <v>1.799999952316284</v>
       </c>
       <c r="C53" t="n">
-        <v>1.69</v>
+        <v>1.720000028610229</v>
       </c>
       <c r="D53" t="n">
-        <v>1.8</v>
+        <v>1.429999947547913</v>
       </c>
       <c r="E53" t="n">
-        <v>5.22</v>
+        <v>4.949999809265137</v>
       </c>
       <c r="F53" t="n">
         <v>0</v>
@@ -1611,16 +1611,16 @@
         </is>
       </c>
       <c r="B54" t="n">
-        <v>1.04</v>
+        <v>1.590000033378601</v>
       </c>
       <c r="C54" t="n">
-        <v>2.27</v>
+        <v>2.680000066757202</v>
       </c>
       <c r="D54" t="n">
-        <v>1.58</v>
+        <v>1.659999966621399</v>
       </c>
       <c r="E54" t="n">
-        <v>4.89</v>
+        <v>5.929999828338623</v>
       </c>
       <c r="F54" t="n">
         <v>0</v>
@@ -1633,16 +1633,16 @@
         </is>
       </c>
       <c r="B55" t="n">
-        <v>2.02</v>
+        <v>2.470000028610229</v>
       </c>
       <c r="C55" t="n">
-        <v>2.21</v>
+        <v>2.630000114440918</v>
       </c>
       <c r="D55" t="n">
-        <v>2.6</v>
+        <v>3</v>
       </c>
       <c r="E55" t="n">
-        <v>6.83</v>
+        <v>8.100000381469727</v>
       </c>
       <c r="F55" t="n">
         <v>1</v>
@@ -1655,16 +1655,16 @@
         </is>
       </c>
       <c r="B56" t="n">
-        <v>1.71</v>
+        <v>1.820000052452087</v>
       </c>
       <c r="C56" t="n">
-        <v>2.77</v>
+        <v>2.359999895095825</v>
       </c>
       <c r="D56" t="n">
-        <v>2.52</v>
+        <v>2.690000057220459</v>
       </c>
       <c r="E56" t="n">
-        <v>7</v>
+        <v>6.869999885559082</v>
       </c>
       <c r="F56" t="n">
         <v>1</v>
@@ -1677,16 +1677,16 @@
         </is>
       </c>
       <c r="B57" t="n">
-        <v>1.21</v>
+        <v>1.389999985694885</v>
       </c>
       <c r="C57" t="n">
-        <v>1.02</v>
+        <v>0.6899999976158142</v>
       </c>
       <c r="D57" t="n">
-        <v>1.06</v>
+        <v>0.5600000023841858</v>
       </c>
       <c r="E57" t="n">
-        <v>3.29</v>
+        <v>2.640000104904175</v>
       </c>
       <c r="F57" t="n">
         <v>0</v>
@@ -1699,16 +1699,16 @@
         </is>
       </c>
       <c r="B58" t="n">
-        <v>1.55</v>
+        <v>1.350000023841858</v>
       </c>
       <c r="C58" t="n">
-        <v>2.18</v>
+        <v>2.359999895095825</v>
       </c>
       <c r="D58" t="n">
-        <v>2.36</v>
+        <v>2.299999952316284</v>
       </c>
       <c r="E58" t="n">
-        <v>6.09</v>
+        <v>6.010000228881836</v>
       </c>
       <c r="F58" t="n">
         <v>1</v>
@@ -1721,19 +1721,19 @@
         </is>
       </c>
       <c r="B59" t="n">
-        <v>1.39</v>
+        <v>2.009999990463257</v>
       </c>
       <c r="C59" t="n">
-        <v>2.35</v>
+        <v>2.019999980926514</v>
       </c>
       <c r="D59" t="n">
-        <v>1.67</v>
+        <v>1.990000009536743</v>
       </c>
       <c r="E59" t="n">
-        <v>5.41</v>
+        <v>6.019999980926514</v>
       </c>
       <c r="F59" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="60">
@@ -1743,16 +1743,16 @@
         </is>
       </c>
       <c r="B60" t="n">
-        <v>1.42</v>
+        <v>1.549999952316284</v>
       </c>
       <c r="C60" t="n">
-        <v>2.3</v>
+        <v>1.950000047683716</v>
       </c>
       <c r="D60" t="n">
-        <v>2.04</v>
+        <v>2.259999990463257</v>
       </c>
       <c r="E60" t="n">
-        <v>5.76</v>
+        <v>5.760000228881836</v>
       </c>
       <c r="F60" t="n">
         <v>0</v>
@@ -1765,16 +1765,16 @@
         </is>
       </c>
       <c r="B61" t="n">
-        <v>1.06</v>
+        <v>1.379999995231628</v>
       </c>
       <c r="C61" t="n">
-        <v>2.25</v>
+        <v>1.840000033378601</v>
       </c>
       <c r="D61" t="n">
-        <v>1.94</v>
+        <v>2.069999933242798</v>
       </c>
       <c r="E61" t="n">
-        <v>5.25</v>
+        <v>5.289999961853027</v>
       </c>
       <c r="F61" t="n">
         <v>0</v>
@@ -1787,16 +1787,16 @@
         </is>
       </c>
       <c r="B62" t="n">
-        <v>1.42</v>
+        <v>1.659999966621399</v>
       </c>
       <c r="C62" t="n">
-        <v>1.84</v>
+        <v>1.659999966621399</v>
       </c>
       <c r="D62" t="n">
-        <v>1.59</v>
+        <v>1.75</v>
       </c>
       <c r="E62" t="n">
-        <v>4.85</v>
+        <v>5.070000171661377</v>
       </c>
       <c r="F62" t="n">
         <v>0</v>
@@ -1809,16 +1809,16 @@
         </is>
       </c>
       <c r="B63" t="n">
-        <v>1.06</v>
+        <v>0.9900000095367432</v>
       </c>
       <c r="C63" t="n">
-        <v>0.91</v>
+        <v>0.6600000262260437</v>
       </c>
       <c r="D63" t="n">
-        <v>1.66</v>
+        <v>1.440000057220459</v>
       </c>
       <c r="E63" t="n">
-        <v>3.63</v>
+        <v>3.089999914169312</v>
       </c>
       <c r="F63" t="n">
         <v>0</v>
@@ -1831,16 +1831,16 @@
         </is>
       </c>
       <c r="B64" t="n">
-        <v>2.55</v>
+        <v>2.049999952316284</v>
       </c>
       <c r="C64" t="n">
-        <v>2.23</v>
+        <v>2.380000114440918</v>
       </c>
       <c r="D64" t="n">
-        <v>2.41</v>
+        <v>2.210000038146973</v>
       </c>
       <c r="E64" t="n">
-        <v>7.19</v>
+        <v>6.639999866485596</v>
       </c>
       <c r="F64" t="n">
         <v>1</v>
@@ -1853,16 +1853,16 @@
         </is>
       </c>
       <c r="B65" t="n">
-        <v>1.76</v>
+        <v>1.899999976158142</v>
       </c>
       <c r="C65" t="n">
-        <v>2.1</v>
+        <v>2.25</v>
       </c>
       <c r="D65" t="n">
-        <v>1.33</v>
+        <v>1.830000042915344</v>
       </c>
       <c r="E65" t="n">
-        <v>5.19</v>
+        <v>5.980000019073486</v>
       </c>
       <c r="F65" t="n">
         <v>0</v>
@@ -1875,16 +1875,16 @@
         </is>
       </c>
       <c r="B66" t="n">
-        <v>1.84</v>
+        <v>2.140000104904175</v>
       </c>
       <c r="C66" t="n">
-        <v>2.17</v>
+        <v>1.940000057220459</v>
       </c>
       <c r="D66" t="n">
-        <v>0.11</v>
+        <v>0.4900000095367432</v>
       </c>
       <c r="E66" t="n">
-        <v>4.12</v>
+        <v>4.570000171661377</v>
       </c>
       <c r="F66" t="n">
         <v>0</v>
@@ -1897,16 +1897,16 @@
         </is>
       </c>
       <c r="B67" t="n">
-        <v>2.66</v>
+        <v>2.509999990463257</v>
       </c>
       <c r="C67" t="n">
-        <v>2.68</v>
+        <v>2.819999933242798</v>
       </c>
       <c r="D67" t="n">
-        <v>2.25</v>
+        <v>2.430000066757202</v>
       </c>
       <c r="E67" t="n">
-        <v>7.59</v>
+        <v>7.760000228881836</v>
       </c>
       <c r="F67" t="n">
         <v>1</v>
@@ -1919,16 +1919,16 @@
         </is>
       </c>
       <c r="B68" t="n">
-        <v>1.02</v>
+        <v>1.409999966621399</v>
       </c>
       <c r="C68" t="n">
-        <v>1.06</v>
+        <v>1.370000004768372</v>
       </c>
       <c r="D68" t="n">
-        <v>1.39</v>
+        <v>1.950000047683716</v>
       </c>
       <c r="E68" t="n">
-        <v>3.47</v>
+        <v>4.730000019073486</v>
       </c>
       <c r="F68" t="n">
         <v>0</v>
@@ -1941,16 +1941,16 @@
         </is>
       </c>
       <c r="B69" t="n">
-        <v>0.89</v>
+        <v>1</v>
       </c>
       <c r="C69" t="n">
-        <v>1.92</v>
+        <v>1.190000057220459</v>
       </c>
       <c r="D69" t="n">
-        <v>0.88</v>
+        <v>0.9399999976158142</v>
       </c>
       <c r="E69" t="n">
-        <v>3.69</v>
+        <v>3.130000114440918</v>
       </c>
       <c r="F69" t="n">
         <v>0</v>
@@ -1963,16 +1963,16 @@
         </is>
       </c>
       <c r="B70" t="n">
-        <v>1.88</v>
+        <v>1.720000028610229</v>
       </c>
       <c r="C70" t="n">
-        <v>1.74</v>
+        <v>1.820000052452087</v>
       </c>
       <c r="D70" t="n">
-        <v>2.3</v>
+        <v>2.269999980926514</v>
       </c>
       <c r="E70" t="n">
-        <v>5.92</v>
+        <v>5.809999942779541</v>
       </c>
       <c r="F70" t="n">
         <v>0</v>
@@ -1985,16 +1985,16 @@
         </is>
       </c>
       <c r="B71" t="n">
-        <v>1.05</v>
+        <v>0.9900000095367432</v>
       </c>
       <c r="C71" t="n">
-        <v>1.58</v>
+        <v>1.320000052452087</v>
       </c>
       <c r="D71" t="n">
-        <v>1.14</v>
+        <v>1.090000033378601</v>
       </c>
       <c r="E71" t="n">
-        <v>3.77</v>
+        <v>3.400000095367432</v>
       </c>
       <c r="F71" t="n">
         <v>0</v>
@@ -2007,16 +2007,16 @@
         </is>
       </c>
       <c r="B72" t="n">
-        <v>1.53</v>
+        <v>1.360000014305115</v>
       </c>
       <c r="C72" t="n">
-        <v>1.95</v>
+        <v>1.779999971389771</v>
       </c>
       <c r="D72" t="n">
-        <v>2.3</v>
+        <v>2.029999971389771</v>
       </c>
       <c r="E72" t="n">
-        <v>5.78</v>
+        <v>5.170000076293945</v>
       </c>
       <c r="F72" t="n">
         <v>0</v>
@@ -2029,16 +2029,16 @@
         </is>
       </c>
       <c r="B73" t="n">
-        <v>1.44</v>
+        <v>1.960000038146973</v>
       </c>
       <c r="C73" t="n">
-        <v>2.71</v>
+        <v>2.589999914169312</v>
       </c>
       <c r="D73" t="n">
-        <v>1.88</v>
+        <v>2.539999961853027</v>
       </c>
       <c r="E73" t="n">
-        <v>6.03</v>
+        <v>7.090000152587891</v>
       </c>
       <c r="F73" t="n">
         <v>1</v>
@@ -2051,19 +2051,19 @@
         </is>
       </c>
       <c r="B74" t="n">
-        <v>1.22</v>
+        <v>1.779999971389771</v>
       </c>
       <c r="C74" t="n">
-        <v>1.97</v>
+        <v>2.150000095367432</v>
       </c>
       <c r="D74" t="n">
-        <v>2</v>
+        <v>2.230000019073486</v>
       </c>
       <c r="E74" t="n">
-        <v>5.19</v>
+        <v>6.159999847412109</v>
       </c>
       <c r="F74" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="75">
@@ -2073,16 +2073,16 @@
         </is>
       </c>
       <c r="B75" t="n">
-        <v>2.04</v>
+        <v>2.369999885559082</v>
       </c>
       <c r="C75" t="n">
-        <v>1.85</v>
+        <v>2.450000047683716</v>
       </c>
       <c r="D75" t="n">
-        <v>2.41</v>
+        <v>2.440000057220459</v>
       </c>
       <c r="E75" t="n">
-        <v>6.3</v>
+        <v>7.260000228881836</v>
       </c>
       <c r="F75" t="n">
         <v>1</v>
@@ -2095,16 +2095,16 @@
         </is>
       </c>
       <c r="B76" t="n">
-        <v>2.1</v>
+        <v>1.879999995231628</v>
       </c>
       <c r="C76" t="n">
-        <v>1.44</v>
+        <v>1.529999971389771</v>
       </c>
       <c r="D76" t="n">
-        <v>2.28</v>
+        <v>1.850000023841858</v>
       </c>
       <c r="E76" t="n">
-        <v>5.82</v>
+        <v>5.260000228881836</v>
       </c>
       <c r="F76" t="n">
         <v>0</v>
@@ -2117,16 +2117,16 @@
         </is>
       </c>
       <c r="B77" t="n">
-        <v>0.67</v>
+        <v>0.5299999713897705</v>
       </c>
       <c r="C77" t="n">
-        <v>1.61</v>
+        <v>1.549999952316284</v>
       </c>
       <c r="D77" t="n">
-        <v>1.5</v>
+        <v>0.8100000023841858</v>
       </c>
       <c r="E77" t="n">
-        <v>3.78</v>
+        <v>2.890000104904175</v>
       </c>
       <c r="F77" t="n">
         <v>0</v>
@@ -2139,16 +2139,16 @@
         </is>
       </c>
       <c r="B78" t="n">
-        <v>1.49</v>
+        <v>1.559999942779541</v>
       </c>
       <c r="C78" t="n">
-        <v>2.1</v>
+        <v>1.799999952316284</v>
       </c>
       <c r="D78" t="n">
-        <v>1.67</v>
+        <v>1.899999976158142</v>
       </c>
       <c r="E78" t="n">
-        <v>5.26</v>
+        <v>5.260000228881836</v>
       </c>
       <c r="F78" t="n">
         <v>0</v>
@@ -2161,19 +2161,19 @@
         </is>
       </c>
       <c r="B79" t="n">
-        <v>2.36</v>
+        <v>1.759999990463257</v>
       </c>
       <c r="C79" t="n">
-        <v>1.79</v>
+        <v>1.889999985694885</v>
       </c>
       <c r="D79" t="n">
-        <v>2.05</v>
+        <v>1.480000019073486</v>
       </c>
       <c r="E79" t="n">
-        <v>6.2</v>
+        <v>5.130000114440918</v>
       </c>
       <c r="F79" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="80">
@@ -2183,19 +2183,19 @@
         </is>
       </c>
       <c r="B80" t="n">
-        <v>2.06</v>
+        <v>1.509999990463257</v>
       </c>
       <c r="C80" t="n">
-        <v>2.06</v>
+        <v>1.929999947547913</v>
       </c>
       <c r="D80" t="n">
-        <v>2.41</v>
+        <v>2.119999885559082</v>
       </c>
       <c r="E80" t="n">
-        <v>6.53</v>
+        <v>5.559999942779541</v>
       </c>
       <c r="F80" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="81">
@@ -2205,16 +2205,16 @@
         </is>
       </c>
       <c r="B81" t="n">
-        <v>1</v>
+        <v>1.370000004768372</v>
       </c>
       <c r="C81" t="n">
-        <v>1.9</v>
+        <v>1.059999942779541</v>
       </c>
       <c r="D81" t="n">
-        <v>1.06</v>
+        <v>0.7400000095367432</v>
       </c>
       <c r="E81" t="n">
-        <v>3.96</v>
+        <v>3.170000076293945</v>
       </c>
       <c r="F81" t="n">
         <v>0</v>
@@ -2227,16 +2227,16 @@
         </is>
       </c>
       <c r="B82" t="n">
-        <v>0.86</v>
+        <v>0.8399999737739563</v>
       </c>
       <c r="C82" t="n">
-        <v>1.95</v>
+        <v>2.119999885559082</v>
       </c>
       <c r="D82" t="n">
-        <v>2.19</v>
+        <v>1.870000004768372</v>
       </c>
       <c r="E82" t="n">
-        <v>5</v>
+        <v>4.829999923706055</v>
       </c>
       <c r="F82" t="n">
         <v>0</v>
@@ -2249,16 +2249,16 @@
         </is>
       </c>
       <c r="B83" t="n">
-        <v>1.19</v>
+        <v>1.549999952316284</v>
       </c>
       <c r="C83" t="n">
-        <v>1.68</v>
+        <v>1.649999976158142</v>
       </c>
       <c r="D83" t="n">
-        <v>1.89</v>
+        <v>1.639999985694885</v>
       </c>
       <c r="E83" t="n">
-        <v>4.76</v>
+        <v>4.840000152587891</v>
       </c>
       <c r="F83" t="n">
         <v>0</v>
@@ -2271,16 +2271,16 @@
         </is>
       </c>
       <c r="B84" t="n">
-        <v>1.54</v>
+        <v>1.450000047683716</v>
       </c>
       <c r="C84" t="n">
-        <v>2.06</v>
+        <v>1.980000019073486</v>
       </c>
       <c r="D84" t="n">
-        <v>1.95</v>
+        <v>2.180000066757202</v>
       </c>
       <c r="E84" t="n">
-        <v>5.55</v>
+        <v>5.610000133514404</v>
       </c>
       <c r="F84" t="n">
         <v>0</v>
@@ -2293,16 +2293,16 @@
         </is>
       </c>
       <c r="B85" t="n">
-        <v>1.71</v>
+        <v>1.899999976158142</v>
       </c>
       <c r="C85" t="n">
-        <v>2.19</v>
+        <v>2.279999971389771</v>
       </c>
       <c r="D85" t="n">
-        <v>2.82</v>
+        <v>2.509999990463257</v>
       </c>
       <c r="E85" t="n">
-        <v>6.72</v>
+        <v>6.690000057220459</v>
       </c>
       <c r="F85" t="n">
         <v>1</v>
@@ -2315,16 +2315,16 @@
         </is>
       </c>
       <c r="B86" t="n">
-        <v>2.03</v>
+        <v>1.710000038146973</v>
       </c>
       <c r="C86" t="n">
-        <v>1.88</v>
+        <v>1.5</v>
       </c>
       <c r="D86" t="n">
-        <v>1.33</v>
+        <v>1.350000023841858</v>
       </c>
       <c r="E86" t="n">
-        <v>5.24</v>
+        <v>4.559999942779541</v>
       </c>
       <c r="F86" t="n">
         <v>0</v>
@@ -2337,16 +2337,16 @@
         </is>
       </c>
       <c r="B87" t="n">
-        <v>1.51</v>
+        <v>1.409999966621399</v>
       </c>
       <c r="C87" t="n">
-        <v>1.74</v>
+        <v>1.809999942779541</v>
       </c>
       <c r="D87" t="n">
-        <v>2.32</v>
+        <v>1.929999947547913</v>
       </c>
       <c r="E87" t="n">
-        <v>5.57</v>
+        <v>5.150000095367432</v>
       </c>
       <c r="F87" t="n">
         <v>0</v>
@@ -2359,16 +2359,16 @@
         </is>
       </c>
       <c r="B88" t="n">
-        <v>1.59</v>
+        <v>1.120000004768372</v>
       </c>
       <c r="C88" t="n">
-        <v>1.4</v>
+        <v>0.9200000166893005</v>
       </c>
       <c r="D88" t="n">
-        <v>0.4</v>
+        <v>0.3300000131130219</v>
       </c>
       <c r="E88" t="n">
-        <v>3.39</v>
+        <v>2.369999885559082</v>
       </c>
       <c r="F88" t="n">
         <v>0</v>
@@ -2381,16 +2381,16 @@
         </is>
       </c>
       <c r="B89" t="n">
-        <v>1.34</v>
+        <v>1</v>
       </c>
       <c r="C89" t="n">
-        <v>0.66</v>
+        <v>0.8199999928474426</v>
       </c>
       <c r="D89" t="n">
-        <v>1.23</v>
+        <v>1.669999957084656</v>
       </c>
       <c r="E89" t="n">
-        <v>3.23</v>
+        <v>3.490000009536743</v>
       </c>
       <c r="F89" t="n">
         <v>0</v>
@@ -2403,16 +2403,16 @@
         </is>
       </c>
       <c r="B90" t="n">
-        <v>1.76</v>
+        <v>1.710000038146973</v>
       </c>
       <c r="C90" t="n">
-        <v>2.16</v>
+        <v>2.5</v>
       </c>
       <c r="D90" t="n">
-        <v>2.69</v>
+        <v>1.960000038146973</v>
       </c>
       <c r="E90" t="n">
-        <v>6.61</v>
+        <v>6.170000076293945</v>
       </c>
       <c r="F90" t="n">
         <v>1</v>
@@ -2425,16 +2425,16 @@
         </is>
       </c>
       <c r="B91" t="n">
-        <v>0.59</v>
+        <v>0.8700000047683716</v>
       </c>
       <c r="C91" t="n">
-        <v>1.69</v>
+        <v>1.360000014305115</v>
       </c>
       <c r="D91" t="n">
-        <v>0.8</v>
+        <v>0.4399999976158142</v>
       </c>
       <c r="E91" t="n">
-        <v>3.08</v>
+        <v>2.670000076293945</v>
       </c>
       <c r="F91" t="n">
         <v>0</v>
@@ -2447,16 +2447,16 @@
         </is>
       </c>
       <c r="B92" t="n">
-        <v>1.6</v>
+        <v>2.140000104904175</v>
       </c>
       <c r="C92" t="n">
-        <v>2.3</v>
+        <v>2.410000085830688</v>
       </c>
       <c r="D92" t="n">
-        <v>0.43</v>
+        <v>1.299999952316284</v>
       </c>
       <c r="E92" t="n">
-        <v>4.33</v>
+        <v>5.849999904632568</v>
       </c>
       <c r="F92" t="n">
         <v>0</v>
@@ -2469,16 +2469,16 @@
         </is>
       </c>
       <c r="B93" t="n">
-        <v>1.07</v>
+        <v>0.9900000095367432</v>
       </c>
       <c r="C93" t="n">
-        <v>2.51</v>
+        <v>2.369999885559082</v>
       </c>
       <c r="D93" t="n">
-        <v>2.12</v>
+        <v>1.960000038146973</v>
       </c>
       <c r="E93" t="n">
-        <v>5.7</v>
+        <v>5.320000171661377</v>
       </c>
       <c r="F93" t="n">
         <v>0</v>
@@ -2491,16 +2491,16 @@
         </is>
       </c>
       <c r="B94" t="n">
-        <v>0.91</v>
+        <v>1.350000023841858</v>
       </c>
       <c r="C94" t="n">
-        <v>2.01</v>
+        <v>1.980000019073486</v>
       </c>
       <c r="D94" t="n">
-        <v>2.22</v>
+        <v>2.490000009536743</v>
       </c>
       <c r="E94" t="n">
-        <v>5.14</v>
+        <v>5.820000171661377</v>
       </c>
       <c r="F94" t="n">
         <v>0</v>
@@ -2513,19 +2513,19 @@
         </is>
       </c>
       <c r="B95" t="n">
-        <v>1.68</v>
+        <v>2.259999990463257</v>
       </c>
       <c r="C95" t="n">
-        <v>1.76</v>
+        <v>1.830000042915344</v>
       </c>
       <c r="D95" t="n">
-        <v>2.22</v>
+        <v>2.259999990463257</v>
       </c>
       <c r="E95" t="n">
-        <v>5.66</v>
+        <v>6.349999904632568</v>
       </c>
       <c r="F95" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="96">
@@ -2535,16 +2535,16 @@
         </is>
       </c>
       <c r="B96" t="n">
-        <v>0.7</v>
+        <v>1.080000042915344</v>
       </c>
       <c r="C96" t="n">
-        <v>1.31</v>
+        <v>1.090000033378601</v>
       </c>
       <c r="D96" t="n">
-        <v>1.4</v>
+        <v>1.289999961853027</v>
       </c>
       <c r="E96" t="n">
-        <v>3.41</v>
+        <v>3.460000038146973</v>
       </c>
       <c r="F96" t="n">
         <v>0</v>
@@ -2557,16 +2557,16 @@
         </is>
       </c>
       <c r="B97" t="n">
-        <v>0.28</v>
+        <v>0.4399999976158142</v>
       </c>
       <c r="C97" t="n">
-        <v>1.62</v>
+        <v>1.240000009536743</v>
       </c>
       <c r="D97" t="n">
-        <v>1.52</v>
+        <v>1.75</v>
       </c>
       <c r="E97" t="n">
-        <v>3.42</v>
+        <v>3.430000066757202</v>
       </c>
       <c r="F97" t="n">
         <v>0</v>
@@ -2579,19 +2579,19 @@
         </is>
       </c>
       <c r="B98" t="n">
-        <v>2.16</v>
+        <v>1.870000004768372</v>
       </c>
       <c r="C98" t="n">
-        <v>1.64</v>
+        <v>1.730000019073486</v>
       </c>
       <c r="D98" t="n">
-        <v>2.54</v>
+        <v>2.309999942779541</v>
       </c>
       <c r="E98" t="n">
-        <v>6.34</v>
+        <v>5.909999847412109</v>
       </c>
       <c r="F98" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="99">
@@ -2601,16 +2601,16 @@
         </is>
       </c>
       <c r="B99" t="n">
-        <v>1.87</v>
+        <v>2.059999942779541</v>
       </c>
       <c r="C99" t="n">
-        <v>2.72</v>
+        <v>2.75</v>
       </c>
       <c r="D99" t="n">
-        <v>2.57</v>
+        <v>2.130000114440918</v>
       </c>
       <c r="E99" t="n">
-        <v>7.16</v>
+        <v>6.940000057220459</v>
       </c>
       <c r="F99" t="n">
         <v>1</v>
@@ -2623,16 +2623,16 @@
         </is>
       </c>
       <c r="B100" t="n">
-        <v>1.66</v>
+        <v>1.110000014305115</v>
       </c>
       <c r="C100" t="n">
-        <v>2.11</v>
+        <v>2.069999933242798</v>
       </c>
       <c r="D100" t="n">
-        <v>1.85</v>
+        <v>1.75</v>
       </c>
       <c r="E100" t="n">
-        <v>5.62</v>
+        <v>4.929999828338623</v>
       </c>
       <c r="F100" t="n">
         <v>0</v>
@@ -2645,16 +2645,16 @@
         </is>
       </c>
       <c r="B101" t="n">
-        <v>1.85</v>
+        <v>1.409999966621399</v>
       </c>
       <c r="C101" t="n">
-        <v>0.98</v>
+        <v>0.8299999833106995</v>
       </c>
       <c r="D101" t="n">
-        <v>0.11</v>
+        <v>0</v>
       </c>
       <c r="E101" t="n">
-        <v>2.94</v>
+        <v>2.240000009536743</v>
       </c>
       <c r="F101" t="n">
         <v>0</v>
@@ -2667,16 +2667,16 @@
         </is>
       </c>
       <c r="B102" t="n">
-        <v>0.67</v>
+        <v>1.129999995231628</v>
       </c>
       <c r="C102" t="n">
-        <v>1.72</v>
+        <v>1.220000028610229</v>
       </c>
       <c r="D102" t="n">
-        <v>1.55</v>
+        <v>0.7900000214576721</v>
       </c>
       <c r="E102" t="n">
-        <v>3.94</v>
+        <v>3.140000104904175</v>
       </c>
       <c r="F102" t="n">
         <v>0</v>
@@ -2689,16 +2689,16 @@
         </is>
       </c>
       <c r="B103" t="n">
-        <v>1.62</v>
+        <v>1.5</v>
       </c>
       <c r="C103" t="n">
-        <v>1</v>
+        <v>0.5799999833106995</v>
       </c>
       <c r="D103" t="n">
-        <v>2.05</v>
+        <v>2.430000066757202</v>
       </c>
       <c r="E103" t="n">
-        <v>4.67</v>
+        <v>4.510000228881836</v>
       </c>
       <c r="F103" t="n">
         <v>0</v>
@@ -2711,16 +2711,16 @@
         </is>
       </c>
       <c r="B104" t="n">
-        <v>2.5</v>
+        <v>2.400000095367432</v>
       </c>
       <c r="C104" t="n">
-        <v>2.22</v>
+        <v>2.400000095367432</v>
       </c>
       <c r="D104" t="n">
-        <v>2.36</v>
+        <v>2.279999971389771</v>
       </c>
       <c r="E104" t="n">
-        <v>7.08</v>
+        <v>7.079999923706055</v>
       </c>
       <c r="F104" t="n">
         <v>1</v>
@@ -2733,16 +2733,16 @@
         </is>
       </c>
       <c r="B105" t="n">
-        <v>1.21</v>
+        <v>0.7400000095367432</v>
       </c>
       <c r="C105" t="n">
-        <v>1.85</v>
+        <v>1.860000014305115</v>
       </c>
       <c r="D105" t="n">
-        <v>2.12</v>
+        <v>1.889999985694885</v>
       </c>
       <c r="E105" t="n">
-        <v>5.18</v>
+        <v>4.489999771118164</v>
       </c>
       <c r="F105" t="n">
         <v>0</v>
@@ -2755,16 +2755,16 @@
         </is>
       </c>
       <c r="B106" t="n">
-        <v>2.06</v>
+        <v>1.919999957084656</v>
       </c>
       <c r="C106" t="n">
-        <v>2.16</v>
+        <v>2.539999961853027</v>
       </c>
       <c r="D106" t="n">
-        <v>2.49</v>
+        <v>2.930000066757202</v>
       </c>
       <c r="E106" t="n">
-        <v>6.71</v>
+        <v>7.389999866485596</v>
       </c>
       <c r="F106" t="n">
         <v>1</v>
@@ -2777,16 +2777,16 @@
         </is>
       </c>
       <c r="B107" t="n">
-        <v>1.74</v>
+        <v>1.620000004768372</v>
       </c>
       <c r="C107" t="n">
-        <v>2.47</v>
+        <v>2.390000104904175</v>
       </c>
       <c r="D107" t="n">
-        <v>2.19</v>
+        <v>2.440000057220459</v>
       </c>
       <c r="E107" t="n">
-        <v>6.4</v>
+        <v>6.449999809265137</v>
       </c>
       <c r="F107" t="n">
         <v>1</v>
@@ -2799,16 +2799,16 @@
         </is>
       </c>
       <c r="B108" t="n">
-        <v>1.22</v>
+        <v>1.370000004768372</v>
       </c>
       <c r="C108" t="n">
-        <v>1.87</v>
+        <v>1.799999952316284</v>
       </c>
       <c r="D108" t="n">
-        <v>1.61</v>
+        <v>2.210000038146973</v>
       </c>
       <c r="E108" t="n">
-        <v>4.7</v>
+        <v>5.380000114440918</v>
       </c>
       <c r="F108" t="n">
         <v>0</v>
@@ -2821,16 +2821,16 @@
         </is>
       </c>
       <c r="B109" t="n">
-        <v>1.94</v>
+        <v>1.490000009536743</v>
       </c>
       <c r="C109" t="n">
-        <v>1.52</v>
+        <v>1.309999942779541</v>
       </c>
       <c r="D109" t="n">
-        <v>2.27</v>
+        <v>2.529999971389771</v>
       </c>
       <c r="E109" t="n">
-        <v>5.73</v>
+        <v>5.329999923706055</v>
       </c>
       <c r="F109" t="n">
         <v>0</v>
@@ -2843,16 +2843,16 @@
         </is>
       </c>
       <c r="B110" t="n">
-        <v>1.18</v>
+        <v>1.429999947547913</v>
       </c>
       <c r="C110" t="n">
-        <v>1.49</v>
+        <v>1.840000033378601</v>
       </c>
       <c r="D110" t="n">
-        <v>2.2</v>
+        <v>2.099999904632568</v>
       </c>
       <c r="E110" t="n">
-        <v>4.87</v>
+        <v>5.369999885559082</v>
       </c>
       <c r="F110" t="n">
         <v>0</v>
@@ -2865,19 +2865,19 @@
         </is>
       </c>
       <c r="B111" t="n">
-        <v>1.95</v>
+        <v>1.779999971389771</v>
       </c>
       <c r="C111" t="n">
-        <v>1.77</v>
+        <v>2.730000019073486</v>
       </c>
       <c r="D111" t="n">
-        <v>2.26</v>
+        <v>2.630000114440918</v>
       </c>
       <c r="E111" t="n">
-        <v>5.98</v>
+        <v>7.139999866485596</v>
       </c>
       <c r="F111" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="112">
@@ -2887,16 +2887,16 @@
         </is>
       </c>
       <c r="B112" t="n">
-        <v>1.74</v>
+        <v>2.269999980926514</v>
       </c>
       <c r="C112" t="n">
-        <v>2.38</v>
+        <v>2.720000028610229</v>
       </c>
       <c r="D112" t="n">
-        <v>2.3</v>
+        <v>2.730000019073486</v>
       </c>
       <c r="E112" t="n">
-        <v>6.42</v>
+        <v>7.71999979019165</v>
       </c>
       <c r="F112" t="n">
         <v>1</v>
@@ -2909,16 +2909,16 @@
         </is>
       </c>
       <c r="B113" t="n">
-        <v>2.08</v>
+        <v>1.649999976158142</v>
       </c>
       <c r="C113" t="n">
-        <v>1.34</v>
+        <v>1.779999971389771</v>
       </c>
       <c r="D113" t="n">
-        <v>2.16</v>
+        <v>2.039999961853027</v>
       </c>
       <c r="E113" t="n">
-        <v>5.58</v>
+        <v>5.46999979019165</v>
       </c>
       <c r="F113" t="n">
         <v>0</v>
@@ -2931,16 +2931,16 @@
         </is>
       </c>
       <c r="B114" t="n">
-        <v>0.87</v>
+        <v>1.320000052452087</v>
       </c>
       <c r="C114" t="n">
-        <v>2.85</v>
+        <v>1.519999980926514</v>
       </c>
       <c r="D114" t="n">
-        <v>0.76</v>
+        <v>1.019999980926514</v>
       </c>
       <c r="E114" t="n">
-        <v>4.48</v>
+        <v>3.859999895095825</v>
       </c>
       <c r="F114" t="n">
         <v>0</v>
@@ -2953,16 +2953,16 @@
         </is>
       </c>
       <c r="B115" t="n">
-        <v>1.85</v>
+        <v>1.809999942779541</v>
       </c>
       <c r="C115" t="n">
-        <v>2.03</v>
+        <v>2.25</v>
       </c>
       <c r="D115" t="n">
-        <v>0.95</v>
+        <v>1.159999966621399</v>
       </c>
       <c r="E115" t="n">
-        <v>4.83</v>
+        <v>5.21999979019165</v>
       </c>
       <c r="F115" t="n">
         <v>0</v>
@@ -2975,19 +2975,19 @@
         </is>
       </c>
       <c r="B116" t="n">
-        <v>1.75</v>
+        <v>1.870000004768372</v>
       </c>
       <c r="C116" t="n">
-        <v>2.14</v>
+        <v>2.75</v>
       </c>
       <c r="D116" t="n">
-        <v>2.01</v>
+        <v>2.279999971389771</v>
       </c>
       <c r="E116" t="n">
-        <v>5.9</v>
+        <v>6.900000095367432</v>
       </c>
       <c r="F116" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="117">
@@ -2997,16 +2997,16 @@
         </is>
       </c>
       <c r="B117" t="n">
-        <v>0.43</v>
+        <v>0.6000000238418579</v>
       </c>
       <c r="C117" t="n">
-        <v>0.48</v>
+        <v>0.5099999904632568</v>
       </c>
       <c r="D117" t="n">
-        <v>1.47</v>
+        <v>1.259999990463257</v>
       </c>
       <c r="E117" t="n">
-        <v>2.38</v>
+        <v>2.369999885559082</v>
       </c>
       <c r="F117" t="n">
         <v>0</v>
@@ -3019,16 +3019,16 @@
         </is>
       </c>
       <c r="B118" t="n">
-        <v>1.1</v>
+        <v>1.440000057220459</v>
       </c>
       <c r="C118" t="n">
-        <v>1.59</v>
+        <v>1.5</v>
       </c>
       <c r="D118" t="n">
-        <v>1.84</v>
+        <v>1.370000004768372</v>
       </c>
       <c r="E118" t="n">
-        <v>4.53</v>
+        <v>4.309999942779541</v>
       </c>
       <c r="F118" t="n">
         <v>0</v>
@@ -3041,16 +3041,16 @@
         </is>
       </c>
       <c r="B119" t="n">
-        <v>1.92</v>
+        <v>1.830000042915344</v>
       </c>
       <c r="C119" t="n">
-        <v>1.85</v>
+        <v>1.830000042915344</v>
       </c>
       <c r="D119" t="n">
-        <v>1.85</v>
+        <v>2.089999914169312</v>
       </c>
       <c r="E119" t="n">
-        <v>5.62</v>
+        <v>5.75</v>
       </c>
       <c r="F119" t="n">
         <v>0</v>
@@ -3063,16 +3063,16 @@
         </is>
       </c>
       <c r="B120" t="n">
-        <v>1.49</v>
+        <v>1.330000042915344</v>
       </c>
       <c r="C120" t="n">
-        <v>1.15</v>
+        <v>1.320000052452087</v>
       </c>
       <c r="D120" t="n">
-        <v>1.23</v>
+        <v>1.5</v>
       </c>
       <c r="E120" t="n">
-        <v>3.87</v>
+        <v>4.150000095367432</v>
       </c>
       <c r="F120" t="n">
         <v>0</v>
@@ -3085,16 +3085,16 @@
         </is>
       </c>
       <c r="B121" t="n">
-        <v>1.84</v>
+        <v>1.669999957084656</v>
       </c>
       <c r="C121" t="n">
-        <v>1.95</v>
+        <v>1.409999966621399</v>
       </c>
       <c r="D121" t="n">
-        <v>2.1</v>
+        <v>2.039999961853027</v>
       </c>
       <c r="E121" t="n">
-        <v>5.89</v>
+        <v>5.119999885559082</v>
       </c>
       <c r="F121" t="n">
         <v>0</v>
@@ -3107,16 +3107,16 @@
         </is>
       </c>
       <c r="B122" t="n">
-        <v>0.83</v>
+        <v>0.2899999916553497</v>
       </c>
       <c r="C122" t="n">
-        <v>0.51</v>
+        <v>0.5</v>
       </c>
       <c r="D122" t="n">
-        <v>0.47</v>
+        <v>0.3199999928474426</v>
       </c>
       <c r="E122" t="n">
-        <v>1.81</v>
+        <v>1.110000014305115</v>
       </c>
       <c r="F122" t="n">
         <v>0</v>
@@ -3129,16 +3129,16 @@
         </is>
       </c>
       <c r="B123" t="n">
-        <v>1.45</v>
+        <v>1.320000052452087</v>
       </c>
       <c r="C123" t="n">
-        <v>1.92</v>
+        <v>1.899999976158142</v>
       </c>
       <c r="D123" t="n">
-        <v>2.07</v>
+        <v>2.190000057220459</v>
       </c>
       <c r="E123" t="n">
-        <v>5.44</v>
+        <v>5.409999847412109</v>
       </c>
       <c r="F123" t="n">
         <v>0</v>
@@ -3151,19 +3151,19 @@
         </is>
       </c>
       <c r="B124" t="n">
-        <v>1.6</v>
+        <v>1.080000042915344</v>
       </c>
       <c r="C124" t="n">
-        <v>2.65</v>
+        <v>2.190000057220459</v>
       </c>
       <c r="D124" t="n">
-        <v>1.81</v>
+        <v>2.119999885559082</v>
       </c>
       <c r="E124" t="n">
-        <v>6.06</v>
+        <v>5.389999866485596</v>
       </c>
       <c r="F124" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="125">
@@ -3173,16 +3173,16 @@
         </is>
       </c>
       <c r="B125" t="n">
-        <v>0.9</v>
+        <v>1.240000009536743</v>
       </c>
       <c r="C125" t="n">
-        <v>1.86</v>
+        <v>2.190000057220459</v>
       </c>
       <c r="D125" t="n">
-        <v>1.83</v>
+        <v>1.830000042915344</v>
       </c>
       <c r="E125" t="n">
-        <v>4.59</v>
+        <v>5.260000228881836</v>
       </c>
       <c r="F125" t="n">
         <v>0</v>
@@ -3195,16 +3195,16 @@
         </is>
       </c>
       <c r="B126" t="n">
-        <v>1.33</v>
+        <v>1.169999957084656</v>
       </c>
       <c r="C126" t="n">
-        <v>1.63</v>
+        <v>2.079999923706055</v>
       </c>
       <c r="D126" t="n">
-        <v>1.75</v>
+        <v>1.870000004768372</v>
       </c>
       <c r="E126" t="n">
-        <v>4.71</v>
+        <v>5.119999885559082</v>
       </c>
       <c r="F126" t="n">
         <v>0</v>
@@ -3217,16 +3217,16 @@
         </is>
       </c>
       <c r="B127" t="n">
-        <v>1.81</v>
+        <v>2.480000019073486</v>
       </c>
       <c r="C127" t="n">
-        <v>2</v>
+        <v>2.289999961853027</v>
       </c>
       <c r="D127" t="n">
-        <v>2.23</v>
+        <v>2.410000085830688</v>
       </c>
       <c r="E127" t="n">
-        <v>6.04</v>
+        <v>7.179999828338623</v>
       </c>
       <c r="F127" t="n">
         <v>1</v>
@@ -3239,19 +3239,19 @@
         </is>
       </c>
       <c r="B128" t="n">
-        <v>1.98</v>
+        <v>2.099999904632568</v>
       </c>
       <c r="C128" t="n">
-        <v>1.56</v>
+        <v>1.850000023841858</v>
       </c>
       <c r="D128" t="n">
-        <v>2.17</v>
+        <v>2.359999895095825</v>
       </c>
       <c r="E128" t="n">
-        <v>5.71</v>
+        <v>6.309999942779541</v>
       </c>
       <c r="F128" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="129">
@@ -3261,16 +3261,16 @@
         </is>
       </c>
       <c r="B129" t="n">
-        <v>2.25</v>
+        <v>1.789999961853027</v>
       </c>
       <c r="C129" t="n">
-        <v>2.44</v>
+        <v>2.460000038146973</v>
       </c>
       <c r="D129" t="n">
-        <v>2.36</v>
+        <v>2.299999952316284</v>
       </c>
       <c r="E129" t="n">
-        <v>7.05</v>
+        <v>6.550000190734863</v>
       </c>
       <c r="F129" t="n">
         <v>1</v>
@@ -3283,16 +3283,16 @@
         </is>
       </c>
       <c r="B130" t="n">
-        <v>0.95</v>
+        <v>0.3300000131130219</v>
       </c>
       <c r="C130" t="n">
-        <v>0.59</v>
+        <v>0.4300000071525574</v>
       </c>
       <c r="D130" t="n">
-        <v>1.38</v>
+        <v>1.320000052452087</v>
       </c>
       <c r="E130" t="n">
-        <v>2.92</v>
+        <v>2.079999923706055</v>
       </c>
       <c r="F130" t="n">
         <v>0</v>
@@ -3305,16 +3305,16 @@
         </is>
       </c>
       <c r="B131" t="n">
-        <v>2.21</v>
+        <v>1.779999971389771</v>
       </c>
       <c r="C131" t="n">
-        <v>1.22</v>
+        <v>1.379999995231628</v>
       </c>
       <c r="D131" t="n">
-        <v>0.11</v>
+        <v>0.3700000047683716</v>
       </c>
       <c r="E131" t="n">
-        <v>3.54</v>
+        <v>3.529999971389771</v>
       </c>
       <c r="F131" t="n">
         <v>0</v>
@@ -3327,16 +3327,16 @@
         </is>
       </c>
       <c r="B132" t="n">
-        <v>1.18</v>
+        <v>1.509999990463257</v>
       </c>
       <c r="C132" t="n">
-        <v>1.47</v>
+        <v>1.610000014305115</v>
       </c>
       <c r="D132" t="n">
-        <v>1.82</v>
+        <v>1.889999985694885</v>
       </c>
       <c r="E132" t="n">
-        <v>4.47</v>
+        <v>5.010000228881836</v>
       </c>
       <c r="F132" t="n">
         <v>0</v>
@@ -3349,19 +3349,19 @@
         </is>
       </c>
       <c r="B133" t="n">
-        <v>1.13</v>
+        <v>1.259999990463257</v>
       </c>
       <c r="C133" t="n">
-        <v>1.92</v>
+        <v>2.210000038146973</v>
       </c>
       <c r="D133" t="n">
-        <v>2.21</v>
+        <v>2.880000114440918</v>
       </c>
       <c r="E133" t="n">
-        <v>5.26</v>
+        <v>6.349999904632568</v>
       </c>
       <c r="F133" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="134">
@@ -3371,16 +3371,16 @@
         </is>
       </c>
       <c r="B134" t="n">
-        <v>0.8100000000000001</v>
+        <v>0.6399999856948853</v>
       </c>
       <c r="C134" t="n">
-        <v>1.47</v>
+        <v>1.549999952316284</v>
       </c>
       <c r="D134" t="n">
-        <v>1.67</v>
+        <v>1.539999961853027</v>
       </c>
       <c r="E134" t="n">
-        <v>3.95</v>
+        <v>3.730000019073486</v>
       </c>
       <c r="F134" t="n">
         <v>0</v>
@@ -3393,19 +3393,19 @@
         </is>
       </c>
       <c r="B135" t="n">
-        <v>1.87</v>
+        <v>1.759999990463257</v>
       </c>
       <c r="C135" t="n">
-        <v>2.72</v>
+        <v>2.369999885559082</v>
       </c>
       <c r="D135" t="n">
-        <v>1.58</v>
+        <v>1.470000028610229</v>
       </c>
       <c r="E135" t="n">
-        <v>6.17</v>
+        <v>5.599999904632568</v>
       </c>
       <c r="F135" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="136">
@@ -3415,16 +3415,16 @@
         </is>
       </c>
       <c r="B136" t="n">
-        <v>1.44</v>
+        <v>0.9599999785423279</v>
       </c>
       <c r="C136" t="n">
-        <v>1.6</v>
+        <v>1.440000057220459</v>
       </c>
       <c r="D136" t="n">
-        <v>2.1</v>
+        <v>1.879999995231628</v>
       </c>
       <c r="E136" t="n">
-        <v>5.14</v>
+        <v>4.28000020980835</v>
       </c>
       <c r="F136" t="n">
         <v>0</v>
@@ -3437,19 +3437,19 @@
         </is>
       </c>
       <c r="B137" t="n">
-        <v>1.15</v>
+        <v>1.669999957084656</v>
       </c>
       <c r="C137" t="n">
-        <v>2.12</v>
+        <v>2.470000028610229</v>
       </c>
       <c r="D137" t="n">
-        <v>2.1</v>
+        <v>2.230000019073486</v>
       </c>
       <c r="E137" t="n">
-        <v>5.37</v>
+        <v>6.369999885559082</v>
       </c>
       <c r="F137" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="138">
@@ -3459,16 +3459,16 @@
         </is>
       </c>
       <c r="B138" t="n">
-        <v>0.67</v>
+        <v>0.4099999964237213</v>
       </c>
       <c r="C138" t="n">
-        <v>1.04</v>
+        <v>1.299999952316284</v>
       </c>
       <c r="D138" t="n">
-        <v>1.96</v>
+        <v>2.170000076293945</v>
       </c>
       <c r="E138" t="n">
-        <v>3.67</v>
+        <v>3.880000114440918</v>
       </c>
       <c r="F138" t="n">
         <v>0</v>
@@ -3481,16 +3481,16 @@
         </is>
       </c>
       <c r="B139" t="n">
-        <v>1.11</v>
+        <v>0.7200000286102295</v>
       </c>
       <c r="C139" t="n">
-        <v>1.41</v>
+        <v>0.9399999976158142</v>
       </c>
       <c r="D139" t="n">
-        <v>1.08</v>
+        <v>1.049999952316284</v>
       </c>
       <c r="E139" t="n">
-        <v>3.6</v>
+        <v>2.710000038146973</v>
       </c>
       <c r="F139" t="n">
         <v>0</v>
@@ -3503,16 +3503,16 @@
         </is>
       </c>
       <c r="B140" t="n">
-        <v>1.41</v>
+        <v>0.9700000286102295</v>
       </c>
       <c r="C140" t="n">
-        <v>1.09</v>
+        <v>1.039999961853027</v>
       </c>
       <c r="D140" t="n">
-        <v>1.36</v>
+        <v>1.210000038146973</v>
       </c>
       <c r="E140" t="n">
-        <v>3.86</v>
+        <v>3.220000028610229</v>
       </c>
       <c r="F140" t="n">
         <v>0</v>
@@ -3525,16 +3525,16 @@
         </is>
       </c>
       <c r="B141" t="n">
-        <v>0.84</v>
+        <v>0.7900000214576721</v>
       </c>
       <c r="C141" t="n">
-        <v>1.42</v>
+        <v>1.919999957084656</v>
       </c>
       <c r="D141" t="n">
-        <v>1.98</v>
+        <v>2.240000009536743</v>
       </c>
       <c r="E141" t="n">
-        <v>4.24</v>
+        <v>4.949999809265137</v>
       </c>
       <c r="F141" t="n">
         <v>0</v>
@@ -3547,19 +3547,19 @@
         </is>
       </c>
       <c r="B142" t="n">
-        <v>1.34</v>
+        <v>1.809999942779541</v>
       </c>
       <c r="C142" t="n">
-        <v>1.6</v>
+        <v>2.150000095367432</v>
       </c>
       <c r="D142" t="n">
-        <v>1.72</v>
+        <v>2.359999895095825</v>
       </c>
       <c r="E142" t="n">
-        <v>4.66</v>
+        <v>6.320000171661377</v>
       </c>
       <c r="F142" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="143">
@@ -3569,16 +3569,16 @@
         </is>
       </c>
       <c r="B143" t="n">
-        <v>0.89</v>
+        <v>0.8600000143051147</v>
       </c>
       <c r="C143" t="n">
-        <v>1.81</v>
+        <v>1.460000038146973</v>
       </c>
       <c r="D143" t="n">
-        <v>0.52</v>
+        <v>0.7799999713897705</v>
       </c>
       <c r="E143" t="n">
-        <v>3.22</v>
+        <v>3.099999904632568</v>
       </c>
       <c r="F143" t="n">
         <v>0</v>
@@ -3591,16 +3591,16 @@
         </is>
       </c>
       <c r="B144" t="n">
-        <v>1.95</v>
+        <v>1.610000014305115</v>
       </c>
       <c r="C144" t="n">
-        <v>1.54</v>
+        <v>1.799999952316284</v>
       </c>
       <c r="D144" t="n">
-        <v>1.94</v>
+        <v>2.049999952316284</v>
       </c>
       <c r="E144" t="n">
-        <v>5.43</v>
+        <v>5.460000038146973</v>
       </c>
       <c r="F144" t="n">
         <v>0</v>
@@ -3613,16 +3613,16 @@
         </is>
       </c>
       <c r="B145" t="n">
-        <v>1.31</v>
+        <v>1.669999957084656</v>
       </c>
       <c r="C145" t="n">
-        <v>1.16</v>
+        <v>0.699999988079071</v>
       </c>
       <c r="D145" t="n">
-        <v>1.17</v>
+        <v>1.350000023841858</v>
       </c>
       <c r="E145" t="n">
-        <v>3.64</v>
+        <v>3.720000028610229</v>
       </c>
       <c r="F145" t="n">
         <v>0</v>
@@ -3635,16 +3635,16 @@
         </is>
       </c>
       <c r="B146" t="n">
-        <v>1.54</v>
+        <v>1.549999952316284</v>
       </c>
       <c r="C146" t="n">
-        <v>1.92</v>
+        <v>2.279999971389771</v>
       </c>
       <c r="D146" t="n">
-        <v>2.01</v>
+        <v>1.950000047683716</v>
       </c>
       <c r="E146" t="n">
-        <v>5.47</v>
+        <v>5.78000020980835</v>
       </c>
       <c r="F146" t="n">
         <v>0</v>
@@ -3657,16 +3657,16 @@
         </is>
       </c>
       <c r="B147" t="n">
-        <v>0.91</v>
+        <v>1.370000004768372</v>
       </c>
       <c r="C147" t="n">
-        <v>1.63</v>
+        <v>2.089999914169312</v>
       </c>
       <c r="D147" t="n">
-        <v>1.62</v>
+        <v>2.180000066757202</v>
       </c>
       <c r="E147" t="n">
-        <v>4.16</v>
+        <v>5.639999866485596</v>
       </c>
       <c r="F147" t="n">
         <v>0</v>
@@ -3679,16 +3679,16 @@
         </is>
       </c>
       <c r="B148" t="n">
-        <v>0.68</v>
+        <v>1.149999976158142</v>
       </c>
       <c r="C148" t="n">
-        <v>1.2</v>
+        <v>1.690000057220459</v>
       </c>
       <c r="D148" t="n">
-        <v>2.19</v>
+        <v>2.009999990463257</v>
       </c>
       <c r="E148" t="n">
-        <v>4.07</v>
+        <v>4.849999904632568</v>
       </c>
       <c r="F148" t="n">
         <v>0</v>
@@ -3701,16 +3701,16 @@
         </is>
       </c>
       <c r="B149" t="n">
-        <v>1.96</v>
+        <v>2.160000085830688</v>
       </c>
       <c r="C149" t="n">
-        <v>1.98</v>
+        <v>2.289999961853027</v>
       </c>
       <c r="D149" t="n">
-        <v>2.56</v>
+        <v>2.160000085830688</v>
       </c>
       <c r="E149" t="n">
-        <v>6.5</v>
+        <v>6.610000133514404</v>
       </c>
       <c r="F149" t="n">
         <v>1</v>
@@ -3723,16 +3723,16 @@
         </is>
       </c>
       <c r="B150" t="n">
-        <v>1.19</v>
+        <v>0.8700000047683716</v>
       </c>
       <c r="C150" t="n">
-        <v>1.81</v>
+        <v>1.399999976158142</v>
       </c>
       <c r="D150" t="n">
-        <v>1.46</v>
+        <v>2.019999980926514</v>
       </c>
       <c r="E150" t="n">
-        <v>4.46</v>
+        <v>4.289999961853027</v>
       </c>
       <c r="F150" t="n">
         <v>0</v>
@@ -3745,16 +3745,16 @@
         </is>
       </c>
       <c r="B151" t="n">
-        <v>1.74</v>
+        <v>1.730000019073486</v>
       </c>
       <c r="C151" t="n">
-        <v>2.25</v>
+        <v>2.039999961853027</v>
       </c>
       <c r="D151" t="n">
-        <v>1.77</v>
+        <v>1.570000052452087</v>
       </c>
       <c r="E151" t="n">
-        <v>5.76</v>
+        <v>5.340000152587891</v>
       </c>
       <c r="F151" t="n">
         <v>0</v>

</xml_diff>